<commit_message>
Update website pages and fix image rendering
</commit_message>
<xml_diff>
--- a/backend/Gryphon_Submissions.xlsx
+++ b/backend/Gryphon_Submissions.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -493,16 +493,62 @@
         <v>I want to talk</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>13/10/2026, 11:11:52 am</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Aniket</v>
+      </c>
+      <c r="C5" t="str">
+        <v>UCIL</v>
+      </c>
+      <c r="D5" t="str">
+        <v>aniket2527@gmail.com</v>
+      </c>
+      <c r="E5" t="str">
+        <v>6207905548</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Training</v>
+      </c>
+      <c r="G5" t="str">
+        <v xml:space="preserve">I want to get training for my custom requirments </v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>13/10/2026, 12:02:22 pm</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Ishika</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v>ishika12378239@gmail.com</v>
+      </c>
+      <c r="E6" t="str">
+        <v>9199204879</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Training</v>
+      </c>
+      <c r="G6" t="str">
+        <v>sgsgshh</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -609,16 +655,51 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>13/10/2026, 11:14:31 am</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Aniket</v>
+      </c>
+      <c r="C4" t="str">
+        <v>UCIL</v>
+      </c>
+      <c r="D4" t="str">
+        <v>AD</v>
+      </c>
+      <c r="E4" t="str">
+        <v>aniket1273@gmail.com</v>
+      </c>
+      <c r="F4" t="str">
+        <v>6207901151</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Cyber Investigation</v>
+      </c>
+      <c r="H4" t="str">
+        <v>5</v>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Online</v>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -684,9 +765,41 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>13/10/2026, 11:08:23 am</v>
+      </c>
+      <c r="B3" t="str">
+        <v xml:space="preserve">Aniket </v>
+      </c>
+      <c r="C3" t="str">
+        <v>UCIL</v>
+      </c>
+      <c r="D3" t="str">
+        <v>AD</v>
+      </c>
+      <c r="E3" t="str">
+        <v>aniket1235@gmail.com</v>
+      </c>
+      <c r="F3" t="str">
+        <v>6207907558</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Custom</v>
+      </c>
+      <c r="H3" t="str">
+        <v>2026-10-31</v>
+      </c>
+      <c r="I3" t="str">
+        <v>3:00 PM</v>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>